<commit_message>
docs(ops): add Discord + Reddit rows to PENDING_MANUAL_TASKS.xlsx
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ops/PENDING_MANUAL_TASKS.xlsx
+++ b/ops/PENDING_MANUAL_TASKS.xlsx
@@ -11,7 +11,7 @@
     <sheet name="What's done" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Manual tasks'!$A$1:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Manual tasks'!$A$1:$I$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1190,8 +1190,115 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="160" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Distribution</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Reddit credentials + sub allow-list</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Reddit account with karma; script-type app</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>1. https://www.reddit.com/prefs/apps → create script app
+2. Copy client_id + client_secret
+3. Append to /opt/football-predict/.env:
+     REDDIT_CLIENT_ID, REDDIT_CLIENT_SECRET,
+     REDDIT_USERNAME, REDDIT_PASSWORD,
+     REDDIT_USER_AGENT='epl-prediction-lab/1.0 by u/&lt;you&gt;',
+     REDDIT_SUBREDDITS='soccerbetting'
+4. docker compose up -d --force-recreate api
+5. Manually run: docker compose exec -T api python scripts/post_reddit_weekly.py
+6. Watch the post; if engagement is good, add SoccerBetting too</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Auto-post Monday 12:00 UTC via weekly.sh. CONSERVATIVE: 1 sub at a time.</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Yes — backend/scripts/post_reddit_weekly.py + weekly.sh wired</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="80" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Distribution</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Promote /discord page to communities</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>30 min</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Outreach bandwidth</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>1. Page is live at predictor.nullshift.sh/discord
+2. Backend fan-out already wired (kind=goal/kickoff/halftime/card/drama/pre_match)
+3. Share /discord URL on football Discord servers + Reddit + Telegram
+4. Server admin pastes their webhook URL → done in 30 sec
+5. Currently 1 webhook registered (test)</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>No bot install, no oAuth — webhook URL is the entire setup.</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Yes — /discord page + /api/discord/register endpoint</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I13"/>
+  <autoFilter ref="A1:I15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>